<commit_message>
Update portfolio_data.xlsx with historical records coloring
Applied blue color (#0066CC) to 45 historical records in the Excel file.
This change demonstrates the fix for color_historical_records() method.

Changes:
- 45 historical records now have Font.color.rgb = "000066CC" (blue)
- 43 current records retain default theme color (black)
- Colors are now properly read by the Portfolio table view

This file was colored using the corrected color_historical_records() method
to validate that the fix works correctly.
</commit_message>
<xml_diff>
--- a/portfolio_data.xlsx
+++ b/portfolio_data.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
     <numFmt numFmtId="165" formatCode="€#,##0.00"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,6 +33,9 @@
       <b val="1"/>
     </font>
     <font/>
+    <font>
+      <color rgb="000066CC"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -62,7 +65,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -71,6 +74,8 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -543,137 +548,140 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Criptovalute</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Trade Republic</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>BTC/EUR</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>BTC/EUR</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>BTC/EUR</t>
         </is>
       </c>
-      <c r="G2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="3" t="n">
+      <c r="G2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="7" t="n">
         <v>45895</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="6" t="n">
         <v>0.010661</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" s="6" t="n">
         <v>93521</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" s="6" t="n">
         <v>997.027381</v>
       </c>
-      <c r="L2" s="3" t="n">
+      <c r="L2" s="7" t="n">
         <v>45932</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M2" s="6" t="n">
         <v>0.010661</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N2" s="6" t="n">
         <v>100725</v>
       </c>
-      <c r="O2" t="n">
+      <c r="O2" s="6" t="n">
         <v>1073.829225</v>
       </c>
-      <c r="Q2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
+      <c r="P2" s="6" t="n"/>
+      <c r="Q2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" s="6" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Criptovalute</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Trade Republic</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>BTC/EUR</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>BTC/EUR</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>BTC/EUR</t>
         </is>
       </c>
-      <c r="G3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" s="3" t="n">
+      <c r="G3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="7" t="n">
         <v>45895</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="6" t="n">
         <v>0.010661</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" s="6" t="n">
         <v>93521</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" s="6" t="n">
         <v>997.027381</v>
       </c>
-      <c r="L3" s="3" t="n">
+      <c r="L3" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M3" t="n">
+      <c r="M3" s="6" t="n">
         <v>0.010661</v>
       </c>
-      <c r="N3" t="n">
+      <c r="N3" s="6" t="n">
         <v>104972.82</v>
       </c>
-      <c r="O3" t="n">
+      <c r="O3" s="6" t="n">
         <v>1119.11523402</v>
       </c>
-      <c r="Q3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" t="inlineStr">
+      <c r="P3" s="6" t="n"/>
+      <c r="Q3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" s="6" t="inlineStr">
         <is>
           <t>UPDATED BY AssetMind</t>
         </is>
@@ -751,137 +759,140 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Fineco_Adv+</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Amundi MSCI Semiconductors UCITS ETF Acc</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>LU1900066033</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>CHIP</t>
         </is>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="H5" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="6" t="n">
         <v>180</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J5" s="6" t="n">
         <v>52.79</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" s="6" t="n">
         <v>9502.200000000001</v>
       </c>
-      <c r="L5" s="3" t="n">
+      <c r="L5" s="7" t="n">
         <v>45932</v>
       </c>
-      <c r="M5" t="n">
+      <c r="M5" s="6" t="n">
         <v>180</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N5" s="6" t="n">
         <v>65.8</v>
       </c>
-      <c r="O5" t="n">
+      <c r="O5" s="6" t="n">
         <v>11844</v>
       </c>
-      <c r="Q5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" t="n">
-        <v>0</v>
-      </c>
+      <c r="P5" s="6" t="n"/>
+      <c r="Q5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="6" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="6" t="n">
         <v>49</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Fineco_Adv+</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Amundi MSCI Semiconductors UCITS ETF Acc</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>LU1900066033</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>CHIP</t>
         </is>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H6" s="3" t="n">
+      <c r="H6" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I6" s="6" t="n">
         <v>180</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J6" s="6" t="n">
         <v>52.79</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K6" s="6" t="n">
         <v>9502.200000000001</v>
       </c>
-      <c r="L6" s="3" t="n">
+      <c r="L6" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M6" t="n">
+      <c r="M6" s="6" t="n">
         <v>180</v>
       </c>
-      <c r="N6" t="n">
+      <c r="N6" s="6" t="n">
         <v>66.63</v>
       </c>
-      <c r="O6" t="n">
+      <c r="O6" s="6" t="n">
         <v>11993.4</v>
       </c>
-      <c r="Q6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" t="inlineStr">
+      <c r="P6" s="6" t="n"/>
+      <c r="Q6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="6" t="inlineStr">
         <is>
           <t>PRICE ALERT - Aggiornato Manualmente</t>
         </is>
@@ -959,137 +970,140 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Fineco_Adv+</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Invesco EQQQ Nasdaq-100 UCITS ETF Acc</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>IE00BFZXGZ54</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>EQAC</t>
         </is>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H8" s="3" t="n">
+      <c r="H8" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I8" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="J8" t="n">
+      <c r="J8" s="6" t="n">
         <v>337.94</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K8" s="6" t="n">
         <v>13517.6</v>
       </c>
-      <c r="L8" s="3" t="n">
+      <c r="L8" s="7" t="n">
         <v>45932</v>
       </c>
-      <c r="M8" t="n">
+      <c r="M8" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="N8" t="n">
+      <c r="N8" s="6" t="n">
         <v>361.95</v>
       </c>
-      <c r="O8" t="n">
+      <c r="O8" s="6" t="n">
         <v>14478</v>
       </c>
-      <c r="Q8" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" t="n">
-        <v>0</v>
-      </c>
-      <c r="S8" t="n">
-        <v>0</v>
-      </c>
+      <c r="P8" s="6" t="n"/>
+      <c r="Q8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Fineco_Adv+</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Invesco EQQQ Nasdaq-100 UCITS ETF Acc</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>IE00BFZXGZ54</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>EQAC</t>
         </is>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H9" s="3" t="n">
+      <c r="H9" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I9" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="J9" t="n">
+      <c r="J9" s="6" t="n">
         <v>337.94</v>
       </c>
-      <c r="K9" t="n">
+      <c r="K9" s="6" t="n">
         <v>13517.6</v>
       </c>
-      <c r="L9" s="3" t="n">
+      <c r="L9" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M9" t="n">
+      <c r="M9" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="N9" t="n">
+      <c r="N9" s="6" t="n">
         <v>362.54</v>
       </c>
-      <c r="O9" t="n">
+      <c r="O9" s="6" t="n">
         <v>14501.6</v>
       </c>
-      <c r="Q9" t="n">
-        <v>0</v>
-      </c>
-      <c r="R9" t="n">
-        <v>0</v>
-      </c>
-      <c r="S9" t="n">
-        <v>0</v>
-      </c>
-      <c r="T9" t="inlineStr">
+      <c r="P9" s="6" t="n"/>
+      <c r="Q9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="6" t="inlineStr">
         <is>
           <t>PRICE ALERT - Aggiornato Manualmente</t>
         </is>
@@ -1167,137 +1181,140 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Fineco_Adv+</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Vanguard FTSE All-World High Div. Yield UCITS ETF Acc</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>IE00BK5BR626</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>VGWE</t>
         </is>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H11" s="3" t="n">
+      <c r="H11" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I11" t="n">
+      <c r="I11" s="6" t="n">
         <v>190</v>
       </c>
-      <c r="J11" t="n">
+      <c r="J11" s="6" t="n">
         <v>70.64</v>
       </c>
-      <c r="K11" t="n">
+      <c r="K11" s="6" t="n">
         <v>13421.6</v>
       </c>
-      <c r="L11" s="3" t="n">
+      <c r="L11" s="7" t="n">
         <v>45932</v>
       </c>
-      <c r="M11" t="n">
+      <c r="M11" s="6" t="n">
         <v>190</v>
       </c>
-      <c r="N11" t="n">
+      <c r="N11" s="6" t="n">
         <v>75.42</v>
       </c>
-      <c r="O11" t="n">
+      <c r="O11" s="6" t="n">
         <v>14329.8</v>
       </c>
-      <c r="Q11" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" t="n">
-        <v>0</v>
-      </c>
+      <c r="P11" s="6" t="n"/>
+      <c r="Q11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="6" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="6" t="n">
         <v>51</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Fineco_Adv+</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Vanguard FTSE All-World High Div. Yield UCITS ETF Acc</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>IE00BK5BR626</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>VGWE</t>
         </is>
       </c>
-      <c r="G12" t="n">
+      <c r="G12" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H12" s="3" t="n">
+      <c r="H12" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I12" t="n">
+      <c r="I12" s="6" t="n">
         <v>190</v>
       </c>
-      <c r="J12" t="n">
+      <c r="J12" s="6" t="n">
         <v>70.64</v>
       </c>
-      <c r="K12" t="n">
+      <c r="K12" s="6" t="n">
         <v>13421.6</v>
       </c>
-      <c r="L12" s="3" t="n">
+      <c r="L12" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M12" t="n">
+      <c r="M12" s="6" t="n">
         <v>190</v>
       </c>
-      <c r="N12" t="n">
+      <c r="N12" s="6" t="n">
         <v>75.68000000000001</v>
       </c>
-      <c r="O12" t="n">
+      <c r="O12" s="6" t="n">
         <v>14379.2</v>
       </c>
-      <c r="Q12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T12" t="inlineStr">
+      <c r="P12" s="6" t="n"/>
+      <c r="Q12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="6" t="inlineStr">
         <is>
           <t>PRICE ALERT - Aggiornato Manualmente</t>
         </is>
@@ -1375,71 +1392,72 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="6" t="n">
         <v>67</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Fineco_Adv+</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>iShares Edge MSCI World Minimum Volatility UCITS ETF USD (Acc)</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>IE00B8FHGS14</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>MVOL.MI</t>
         </is>
       </c>
-      <c r="G14" t="n">
+      <c r="G14" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H14" s="3" t="n">
+      <c r="H14" s="7" t="n">
         <v>41243</v>
       </c>
-      <c r="I14" t="n">
+      <c r="I14" s="6" t="n">
         <v>230</v>
       </c>
-      <c r="J14" t="n">
+      <c r="J14" s="6" t="n">
         <v>62.57</v>
       </c>
-      <c r="K14" t="n">
+      <c r="K14" s="6" t="n">
         <v>14391.1</v>
       </c>
-      <c r="L14" s="3" t="n">
+      <c r="L14" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M14" t="n">
+      <c r="M14" s="6" t="n">
         <v>230</v>
       </c>
-      <c r="N14" t="n">
+      <c r="N14" s="6" t="n">
         <v>62.85</v>
       </c>
-      <c r="O14" t="n">
+      <c r="O14" s="6" t="n">
         <v>14455.5</v>
       </c>
-      <c r="Q14" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" t="n">
-        <v>0</v>
-      </c>
-      <c r="T14" t="inlineStr">
+      <c r="P14" s="6" t="n"/>
+      <c r="Q14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="6" t="inlineStr">
         <is>
           <t>Aggiornato Manualmente</t>
         </is>
@@ -1517,142 +1535,144 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Fineco_auto</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Amundi IS MSCI Europe UCITS ETF DR</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>LU1437015735</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>CEU2</t>
         </is>
       </c>
-      <c r="G16" t="n">
+      <c r="G16" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H16" s="3" t="n">
+      <c r="H16" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I16" s="6" t="n">
         <v>75</v>
       </c>
-      <c r="J16" t="n">
+      <c r="J16" s="6" t="n">
         <v>102.52</v>
       </c>
-      <c r="K16" t="n">
+      <c r="K16" s="6" t="n">
         <v>7689</v>
       </c>
-      <c r="L16" s="3" t="n">
+      <c r="L16" s="7" t="n">
         <v>45931</v>
       </c>
-      <c r="M16" t="n">
+      <c r="M16" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="N16" t="n">
+      <c r="N16" s="6" t="n">
         <v>105.817001</v>
       </c>
-      <c r="O16" t="n">
+      <c r="O16" s="6" t="n">
         <v>529.085005</v>
       </c>
-      <c r="Q16" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" t="n">
-        <v>0</v>
-      </c>
-      <c r="S16" t="n">
-        <v>0</v>
-      </c>
-      <c r="T16" t="inlineStr">
+      <c r="P16" s="6" t="n"/>
+      <c r="Q16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" s="6" t="inlineStr">
         <is>
           <t>Autogestito | UPDATED BY AssetMind</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="6" t="n">
         <v>52</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Fineco_auto</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>Amundi IS MSCI Europe UCITS ETF DR</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>LU1437015735</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>CEU2</t>
         </is>
       </c>
-      <c r="G17" t="n">
+      <c r="G17" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H17" s="3" t="n">
+      <c r="H17" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I17" t="n">
+      <c r="I17" s="6" t="n">
         <v>75</v>
       </c>
-      <c r="J17" t="n">
+      <c r="J17" s="6" t="n">
         <v>102.52</v>
       </c>
-      <c r="K17" t="n">
+      <c r="K17" s="6" t="n">
         <v>7689</v>
       </c>
-      <c r="L17" s="3" t="n">
+      <c r="L17" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M17" t="n">
+      <c r="M17" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="N17" t="n">
+      <c r="N17" s="6" t="n">
         <v>106.867996</v>
       </c>
-      <c r="O17" t="n">
+      <c r="O17" s="6" t="n">
         <v>534.33998</v>
       </c>
-      <c r="Q17" t="n">
-        <v>0</v>
-      </c>
-      <c r="R17" t="n">
-        <v>0</v>
-      </c>
-      <c r="S17" t="n">
-        <v>0</v>
-      </c>
-      <c r="T17" t="inlineStr">
+      <c r="P17" s="6" t="n"/>
+      <c r="Q17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" s="6" t="inlineStr">
         <is>
           <t>UPDATED BY AssetMind</t>
         </is>
@@ -1730,142 +1750,144 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>Fineco_auto</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>ETF ISHS EUR INF-LKD</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>IE00B0M62X26</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>IBCI.AS</t>
         </is>
       </c>
-      <c r="G19" t="n">
+      <c r="G19" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H19" s="3" t="n">
+      <c r="H19" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I19" t="n">
+      <c r="I19" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="J19" t="n">
+      <c r="J19" s="6" t="n">
         <v>226.95</v>
       </c>
-      <c r="K19" t="n">
+      <c r="K19" s="6" t="n">
         <v>10212.75</v>
       </c>
-      <c r="L19" s="3" t="n">
+      <c r="L19" s="7" t="n">
         <v>45931</v>
       </c>
-      <c r="M19" t="n">
+      <c r="M19" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="N19" t="n">
+      <c r="N19" s="6" t="n">
         <v>230.050003</v>
       </c>
-      <c r="O19" t="n">
+      <c r="O19" s="6" t="n">
         <v>10352.250135</v>
       </c>
-      <c r="Q19" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" t="n">
-        <v>0</v>
-      </c>
-      <c r="S19" t="n">
-        <v>0</v>
-      </c>
-      <c r="T19" t="inlineStr">
+      <c r="P19" s="6" t="n"/>
+      <c r="Q19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" s="6" t="inlineStr">
         <is>
           <t>Autogestito | UPDATED BY AssetMind</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" s="6" t="n">
         <v>53</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>Fineco_auto</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>ETF ISHS EUR INF-LKD</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>IE00B0M62X26</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>IBCI.AS</t>
         </is>
       </c>
-      <c r="G20" t="n">
+      <c r="G20" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H20" s="3" t="n">
+      <c r="H20" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I20" t="n">
+      <c r="I20" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="J20" t="n">
+      <c r="J20" s="6" t="n">
         <v>226.95</v>
       </c>
-      <c r="K20" t="n">
+      <c r="K20" s="6" t="n">
         <v>10212.75</v>
       </c>
-      <c r="L20" s="3" t="n">
+      <c r="L20" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M20" t="n">
+      <c r="M20" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="N20" t="n">
+      <c r="N20" s="6" t="n">
         <v>230.509995</v>
       </c>
-      <c r="O20" t="n">
+      <c r="O20" s="6" t="n">
         <v>10372.949775</v>
       </c>
-      <c r="Q20" t="n">
-        <v>0</v>
-      </c>
-      <c r="R20" t="n">
-        <v>0</v>
-      </c>
-      <c r="S20" t="n">
-        <v>0</v>
-      </c>
-      <c r="T20" t="inlineStr">
+      <c r="P20" s="6" t="n"/>
+      <c r="Q20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" s="6" t="inlineStr">
         <is>
           <t>UPDATED BY AssetMind</t>
         </is>
@@ -1943,142 +1965,144 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>Fineco_auto</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>FAM ARTIF INTEL CL A</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>IE000QU8JEH5</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>AI4U.MI</t>
         </is>
       </c>
-      <c r="G22" t="n">
+      <c r="G22" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H22" s="3" t="n">
+      <c r="H22" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I22" t="n">
+      <c r="I22" s="6" t="n">
         <v>122</v>
       </c>
-      <c r="J22" t="n">
+      <c r="J22" s="6" t="n">
         <v>133.38836</v>
       </c>
-      <c r="K22" t="n">
+      <c r="K22" s="6" t="n">
         <v>16273.37992</v>
       </c>
-      <c r="L22" s="3" t="n">
+      <c r="L22" s="7" t="n">
         <v>45931</v>
       </c>
-      <c r="M22" t="n">
+      <c r="M22" s="6" t="n">
         <v>122</v>
       </c>
-      <c r="N22" t="n">
+      <c r="N22" s="6" t="n">
         <v>142.839996</v>
       </c>
-      <c r="O22" t="n">
+      <c r="O22" s="6" t="n">
         <v>17426.479512</v>
       </c>
-      <c r="Q22" t="n">
-        <v>0</v>
-      </c>
-      <c r="R22" t="n">
-        <v>0</v>
-      </c>
-      <c r="S22" t="n">
-        <v>0</v>
-      </c>
-      <c r="T22" t="inlineStr">
+      <c r="P22" s="6" t="n"/>
+      <c r="Q22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T22" s="6" t="inlineStr">
         <is>
           <t>Autogestito | UPDATED BY AssetMind</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="A23" s="6" t="n">
         <v>54</v>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Fineco_auto</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>FAM ARTIF INTEL CL A</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>IE000QU8JEH5</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>AI4U.MI</t>
         </is>
       </c>
-      <c r="G23" t="n">
+      <c r="G23" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H23" s="3" t="n">
+      <c r="H23" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I23" t="n">
+      <c r="I23" s="6" t="n">
         <v>122</v>
       </c>
-      <c r="J23" t="n">
+      <c r="J23" s="6" t="n">
         <v>133.38836</v>
       </c>
-      <c r="K23" t="n">
+      <c r="K23" s="6" t="n">
         <v>16273.37992</v>
       </c>
-      <c r="L23" s="3" t="n">
+      <c r="L23" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M23" t="n">
+      <c r="M23" s="6" t="n">
         <v>122</v>
       </c>
-      <c r="N23" t="n">
+      <c r="N23" s="6" t="n">
         <v>145.089996</v>
       </c>
-      <c r="O23" t="n">
+      <c r="O23" s="6" t="n">
         <v>17700.979512</v>
       </c>
-      <c r="Q23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R23" t="n">
-        <v>0</v>
-      </c>
-      <c r="S23" t="n">
-        <v>0</v>
-      </c>
-      <c r="T23" t="inlineStr">
+      <c r="P23" s="6" t="n"/>
+      <c r="Q23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T23" s="6" t="inlineStr">
         <is>
           <t>UPDATED BY AssetMind</t>
         </is>
@@ -2156,142 +2180,144 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
+      <c r="A25" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>Fineco_auto</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>ISH CO GLB EUR-AC</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>IE00BDBRDM35</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>AGGH.MI</t>
         </is>
       </c>
-      <c r="G25" t="n">
+      <c r="G25" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H25" s="3" t="n">
+      <c r="H25" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I25" t="n">
+      <c r="I25" s="6" t="n">
         <v>4200</v>
       </c>
-      <c r="J25" t="n">
+      <c r="J25" s="6" t="n">
         <v>4.818</v>
       </c>
-      <c r="K25" t="n">
+      <c r="K25" s="6" t="n">
         <v>20235.6</v>
       </c>
-      <c r="L25" s="3" t="n">
+      <c r="L25" s="7" t="n">
         <v>45931</v>
       </c>
-      <c r="M25" t="n">
+      <c r="M25" s="6" t="n">
         <v>4200</v>
       </c>
-      <c r="N25" t="n">
+      <c r="N25" s="6" t="n">
         <v>4.9215</v>
       </c>
-      <c r="O25" t="n">
+      <c r="O25" s="6" t="n">
         <v>20670.3</v>
       </c>
-      <c r="Q25" t="n">
-        <v>0</v>
-      </c>
-      <c r="R25" t="n">
-        <v>0</v>
-      </c>
-      <c r="S25" t="n">
-        <v>0</v>
-      </c>
-      <c r="T25" t="inlineStr">
+      <c r="P25" s="6" t="n"/>
+      <c r="Q25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T25" s="6" t="inlineStr">
         <is>
           <t>Autogestito | UPDATED BY AssetMind</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="n">
+      <c r="A26" s="6" t="n">
         <v>55</v>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>Fineco_auto</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>ISH CO GLB EUR-AC</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>IE00BDBRDM35</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>AGGH.MI</t>
         </is>
       </c>
-      <c r="G26" t="n">
+      <c r="G26" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H26" s="3" t="n">
+      <c r="H26" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I26" t="n">
+      <c r="I26" s="6" t="n">
         <v>4200</v>
       </c>
-      <c r="J26" t="n">
+      <c r="J26" s="6" t="n">
         <v>4.818</v>
       </c>
-      <c r="K26" t="n">
+      <c r="K26" s="6" t="n">
         <v>20235.6</v>
       </c>
-      <c r="L26" s="3" t="n">
+      <c r="L26" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M26" t="n">
+      <c r="M26" s="6" t="n">
         <v>4200</v>
       </c>
-      <c r="N26" t="n">
+      <c r="N26" s="6" t="n">
         <v>4.93</v>
       </c>
-      <c r="O26" t="n">
+      <c r="O26" s="6" t="n">
         <v>20706</v>
       </c>
-      <c r="Q26" t="n">
-        <v>0</v>
-      </c>
-      <c r="R26" t="n">
-        <v>0</v>
-      </c>
-      <c r="S26" t="n">
-        <v>0</v>
-      </c>
-      <c r="T26" t="inlineStr">
+      <c r="P26" s="6" t="n"/>
+      <c r="Q26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T26" s="6" t="inlineStr">
         <is>
           <t>UPDATED BY AssetMind</t>
         </is>
@@ -2369,137 +2395,140 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="n">
+      <c r="A28" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>Fineco_auto</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>Vanguard S&amp;P 500 UCITS ETF (USD) Dis</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>IE00B3XXRP09</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>VUSA.MI</t>
         </is>
       </c>
-      <c r="G28" t="n">
+      <c r="G28" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H28" s="3" t="n">
+      <c r="H28" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I28" t="n">
+      <c r="I28" s="6" t="n">
         <v>210</v>
       </c>
-      <c r="J28" t="n">
+      <c r="J28" s="6" t="n">
         <v>33.02</v>
       </c>
-      <c r="K28" t="n">
+      <c r="K28" s="6" t="n">
         <v>6934.200000000001</v>
       </c>
-      <c r="L28" s="3" t="n">
+      <c r="L28" s="7" t="n">
         <v>45932</v>
       </c>
-      <c r="M28" t="n">
+      <c r="M28" s="6" t="n">
         <v>425</v>
       </c>
-      <c r="N28" t="n">
+      <c r="N28" s="6" t="n">
         <v>108.42</v>
       </c>
-      <c r="O28" t="n">
+      <c r="O28" s="6" t="n">
         <v>46078.5</v>
       </c>
-      <c r="Q28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R28" t="n">
-        <v>0</v>
-      </c>
-      <c r="S28" t="n">
-        <v>0</v>
-      </c>
+      <c r="P28" s="6" t="n"/>
+      <c r="Q28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T28" s="6" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" t="n">
+      <c r="A29" s="6" t="n">
         <v>56</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>Fineco_auto</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>Vanguard S&amp;P 500 UCITS ETF (USD) Dis</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>IE00B3XXRP09</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>VUSA.MI</t>
         </is>
       </c>
-      <c r="G29" t="n">
+      <c r="G29" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H29" s="3" t="n">
+      <c r="H29" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I29" t="n">
+      <c r="I29" s="6" t="n">
         <v>210</v>
       </c>
-      <c r="J29" t="n">
+      <c r="J29" s="6" t="n">
         <v>33.02</v>
       </c>
-      <c r="K29" t="n">
+      <c r="K29" s="6" t="n">
         <v>6934.200000000001</v>
       </c>
-      <c r="L29" s="3" t="n">
+      <c r="L29" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M29" t="n">
+      <c r="M29" s="6" t="n">
         <v>425</v>
       </c>
-      <c r="N29" t="n">
+      <c r="N29" s="6" t="n">
         <v>108.769997</v>
       </c>
-      <c r="O29" t="n">
+      <c r="O29" s="6" t="n">
         <v>46227.248725</v>
       </c>
-      <c r="Q29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R29" t="n">
-        <v>0</v>
-      </c>
-      <c r="S29" t="n">
-        <v>0</v>
-      </c>
-      <c r="T29" t="inlineStr">
+      <c r="P29" s="6" t="n"/>
+      <c r="Q29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T29" s="6" t="inlineStr">
         <is>
           <t>UPDATED BY AssetMind</t>
         </is>
@@ -2577,137 +2606,140 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="n">
+      <c r="A31" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>Fineco_auto</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>IE00B4L5Y983</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>SWDA.MI</t>
         </is>
       </c>
-      <c r="G31" t="n">
+      <c r="G31" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H31" s="3" t="n">
+      <c r="H31" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I31" t="n">
+      <c r="I31" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="J31" t="n">
+      <c r="J31" s="6" t="n">
         <v>99.86</v>
       </c>
-      <c r="K31" t="n">
+      <c r="K31" s="6" t="n">
         <v>39944</v>
       </c>
-      <c r="L31" s="3" t="n">
+      <c r="L31" s="7" t="n">
         <v>45932</v>
       </c>
-      <c r="M31" t="n">
+      <c r="M31" s="6" t="n">
         <v>450</v>
       </c>
-      <c r="N31" t="n">
+      <c r="N31" s="6" t="n">
         <v>108.36</v>
       </c>
-      <c r="O31" t="n">
+      <c r="O31" s="6" t="n">
         <v>48762</v>
       </c>
-      <c r="Q31" t="n">
-        <v>0</v>
-      </c>
-      <c r="R31" t="n">
-        <v>0</v>
-      </c>
-      <c r="S31" t="n">
-        <v>0</v>
-      </c>
+      <c r="P31" s="6" t="n"/>
+      <c r="Q31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T31" s="6" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" t="n">
+      <c r="A32" s="6" t="n">
         <v>57</v>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>Fineco_auto</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>IE00B4L5Y983</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>SWDA.MI</t>
         </is>
       </c>
-      <c r="G32" t="n">
+      <c r="G32" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H32" s="3" t="n">
+      <c r="H32" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I32" t="n">
+      <c r="I32" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="J32" t="n">
+      <c r="J32" s="6" t="n">
         <v>99.86</v>
       </c>
-      <c r="K32" t="n">
+      <c r="K32" s="6" t="n">
         <v>39944</v>
       </c>
-      <c r="L32" s="3" t="n">
+      <c r="L32" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M32" t="n">
+      <c r="M32" s="6" t="n">
         <v>450</v>
       </c>
-      <c r="N32" t="n">
+      <c r="N32" s="6" t="n">
         <v>108.870003</v>
       </c>
-      <c r="O32" t="n">
+      <c r="O32" s="6" t="n">
         <v>48991.50135</v>
       </c>
-      <c r="Q32" t="n">
-        <v>0</v>
-      </c>
-      <c r="R32" t="n">
-        <v>0</v>
-      </c>
-      <c r="S32" t="n">
-        <v>0</v>
-      </c>
-      <c r="T32" t="inlineStr">
+      <c r="P32" s="6" t="n"/>
+      <c r="Q32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T32" s="6" t="inlineStr">
         <is>
           <t>UPDATED BY AssetMind</t>
         </is>
@@ -2785,142 +2817,144 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="n">
+      <c r="A34" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>Mediobanca_auto</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>IS CR 500 USD-AC EUR</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>IE00B5BMR087</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <t>SXR8</t>
         </is>
       </c>
-      <c r="G34" t="n">
+      <c r="G34" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H34" s="3" t="n">
+      <c r="H34" s="7" t="n">
         <v>45610</v>
       </c>
-      <c r="I34" t="n">
+      <c r="I34" s="6" t="n">
         <v>60</v>
       </c>
-      <c r="J34" t="n">
+      <c r="J34" s="6" t="n">
         <v>549.0410000000001</v>
       </c>
-      <c r="K34" t="n">
+      <c r="K34" s="6" t="n">
         <v>32942.46000000001</v>
       </c>
-      <c r="L34" s="3" t="n">
+      <c r="L34" s="7" t="n">
         <v>45932</v>
       </c>
-      <c r="M34" t="n">
+      <c r="M34" s="6" t="n">
         <v>60</v>
       </c>
-      <c r="N34" t="n">
+      <c r="N34" s="6" t="n">
         <v>611.61</v>
       </c>
-      <c r="O34" t="n">
+      <c r="O34" s="6" t="n">
         <v>36696.6</v>
       </c>
-      <c r="Q34" t="n">
-        <v>0</v>
-      </c>
-      <c r="R34" t="n">
-        <v>0</v>
-      </c>
-      <c r="S34" t="n">
-        <v>0</v>
-      </c>
-      <c r="T34" t="inlineStr">
+      <c r="P34" s="6" t="n"/>
+      <c r="Q34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T34" s="6" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="n">
+      <c r="A35" s="6" t="n">
         <v>58</v>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>Mediobanca_auto</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>IS CR 500 USD-AC EUR</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="6" t="inlineStr">
         <is>
           <t>IE00B5BMR087</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="6" t="inlineStr">
         <is>
           <t>SXR8</t>
         </is>
       </c>
-      <c r="G35" t="n">
+      <c r="G35" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H35" s="3" t="n">
+      <c r="H35" s="7" t="n">
         <v>45610</v>
       </c>
-      <c r="I35" t="n">
+      <c r="I35" s="6" t="n">
         <v>60</v>
       </c>
-      <c r="J35" t="n">
+      <c r="J35" s="6" t="n">
         <v>563.9015000000001</v>
       </c>
-      <c r="K35" t="n">
+      <c r="K35" s="6" t="n">
         <v>33834.09</v>
       </c>
-      <c r="L35" s="3" t="n">
+      <c r="L35" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M35" t="n">
+      <c r="M35" s="6" t="n">
         <v>60</v>
       </c>
-      <c r="N35" t="n">
+      <c r="N35" s="6" t="n">
         <v>613.7</v>
       </c>
-      <c r="O35" t="n">
+      <c r="O35" s="6" t="n">
         <v>36822</v>
       </c>
-      <c r="Q35" t="n">
-        <v>0</v>
-      </c>
-      <c r="R35" t="n">
-        <v>0</v>
-      </c>
-      <c r="S35" t="n">
-        <v>0</v>
-      </c>
-      <c r="T35" t="inlineStr">
+      <c r="P35" s="6" t="n"/>
+      <c r="Q35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" s="6" t="inlineStr">
         <is>
           <t>Aggiornato Manualmente | PRICE ALERT</t>
         </is>
@@ -2998,71 +3032,72 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="n">
+      <c r="A37" s="6" t="n">
         <v>68</v>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>Trade Republic</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>Core MSCI EM IMI USD (Acc)</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="6" t="inlineStr">
         <is>
           <t>IE00BKM4GZ66</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" s="6" t="inlineStr">
         <is>
           <t>EIMI.MI</t>
         </is>
       </c>
-      <c r="G37" t="n">
+      <c r="G37" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H37" s="3" t="n">
+      <c r="H37" s="7" t="n">
         <v>41789</v>
       </c>
-      <c r="I37" t="n">
+      <c r="I37" s="6" t="n">
         <v>104.740071</v>
       </c>
-      <c r="J37" t="n">
+      <c r="J37" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="K37" t="n">
+      <c r="K37" s="6" t="n">
         <v>3142.20213</v>
       </c>
-      <c r="L37" s="3" t="n">
+      <c r="L37" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M37" t="n">
+      <c r="M37" s="6" t="n">
         <v>638.274909</v>
       </c>
-      <c r="N37" t="n">
+      <c r="N37" s="6" t="n">
         <v>37.32</v>
       </c>
-      <c r="O37" t="n">
+      <c r="O37" s="6" t="n">
         <v>23820.41960388</v>
       </c>
-      <c r="Q37" t="n">
-        <v>0</v>
-      </c>
-      <c r="R37" t="n">
-        <v>0</v>
-      </c>
-      <c r="S37" t="n">
-        <v>0</v>
-      </c>
-      <c r="T37" t="inlineStr">
+      <c r="P37" s="6" t="n"/>
+      <c r="Q37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T37" s="6" t="inlineStr">
         <is>
           <t>Aggiornato Manualmente</t>
         </is>
@@ -3140,142 +3175,144 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="n">
+      <c r="A39" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>Trade Republic</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>Core MSCI World USD (Acc)</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="6" t="inlineStr">
         <is>
           <t>IE000BI8OT95</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="6" t="inlineStr">
         <is>
           <t>MWRD</t>
         </is>
       </c>
-      <c r="G39" t="n">
+      <c r="G39" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H39" s="3" t="n">
+      <c r="H39" s="7" t="n">
         <v>45904</v>
       </c>
-      <c r="I39" t="n">
+      <c r="I39" s="6" t="n">
         <v>4.685596</v>
       </c>
-      <c r="J39" t="n">
+      <c r="J39" s="6" t="n">
         <v>130.014</v>
       </c>
-      <c r="K39" t="n">
+      <c r="K39" s="6" t="n">
         <v>609.1930783440001</v>
       </c>
-      <c r="L39" s="3" t="n">
+      <c r="L39" s="7" t="n">
         <v>45931</v>
       </c>
-      <c r="M39" t="n">
+      <c r="M39" s="6" t="n">
         <v>4.685596</v>
       </c>
-      <c r="N39" t="n">
+      <c r="N39" s="6" t="n">
         <v>135.662003</v>
       </c>
-      <c r="O39" t="n">
+      <c r="O39" s="6" t="n">
         <v>635.657338608788</v>
       </c>
-      <c r="Q39" t="n">
-        <v>0</v>
-      </c>
-      <c r="R39" t="n">
-        <v>0</v>
-      </c>
-      <c r="S39" t="n">
-        <v>0</v>
-      </c>
-      <c r="T39" t="inlineStr">
+      <c r="P39" s="6" t="n"/>
+      <c r="Q39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T39" s="6" t="inlineStr">
         <is>
           <t>Autogestito | UPDATED BY AssetMind</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="n">
+      <c r="A40" s="6" t="n">
         <v>61</v>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>Trade Republic</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>Core MSCI World USD (Acc)</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>IE000BI8OT95</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <t>MWRD</t>
         </is>
       </c>
-      <c r="G40" t="n">
+      <c r="G40" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H40" s="3" t="n">
+      <c r="H40" s="7" t="n">
         <v>45904</v>
       </c>
-      <c r="I40" t="n">
+      <c r="I40" s="6" t="n">
         <v>4.685596</v>
       </c>
-      <c r="J40" t="n">
+      <c r="J40" s="6" t="n">
         <v>130.014</v>
       </c>
-      <c r="K40" t="n">
+      <c r="K40" s="6" t="n">
         <v>609.1930783440001</v>
       </c>
-      <c r="L40" s="3" t="n">
+      <c r="L40" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M40" t="n">
+      <c r="M40" s="6" t="n">
         <v>4.685596</v>
       </c>
-      <c r="N40" t="n">
+      <c r="N40" s="6" t="n">
         <v>136.712006</v>
       </c>
-      <c r="O40" t="n">
+      <c r="O40" s="6" t="n">
         <v>640.577228465576</v>
       </c>
-      <c r="Q40" t="n">
-        <v>0</v>
-      </c>
-      <c r="R40" t="n">
-        <v>0</v>
-      </c>
-      <c r="S40" t="n">
-        <v>0</v>
-      </c>
-      <c r="T40" t="inlineStr">
+      <c r="P40" s="6" t="n"/>
+      <c r="Q40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T40" s="6" t="inlineStr">
         <is>
           <t>UPDATED BY AssetMind</t>
         </is>
@@ -3353,137 +3390,140 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="n">
+      <c r="A42" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>Trade Republic</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>Core MSCI World USD (Acc)</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E42" s="6" t="inlineStr">
         <is>
           <t>IE00B4L5Y983</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" s="6" t="inlineStr">
         <is>
           <t>A0RPWH</t>
         </is>
       </c>
-      <c r="G42" t="n">
+      <c r="G42" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H42" s="3" t="n">
+      <c r="H42" s="7" t="n">
         <v>45895</v>
       </c>
-      <c r="I42" t="n">
+      <c r="I42" s="6" t="n">
         <v>104.740071</v>
       </c>
-      <c r="J42" t="n">
+      <c r="J42" s="6" t="n">
         <v>85.94</v>
       </c>
-      <c r="K42" t="n">
+      <c r="K42" s="6" t="n">
         <v>9001.361701739999</v>
       </c>
-      <c r="L42" s="3" t="n">
+      <c r="L42" s="7" t="n">
         <v>45932</v>
       </c>
-      <c r="M42" t="n">
+      <c r="M42" s="6" t="n">
         <v>104.740071</v>
       </c>
-      <c r="N42" t="n">
+      <c r="N42" s="6" t="n">
         <v>108.39</v>
       </c>
-      <c r="O42" t="n">
+      <c r="O42" s="6" t="n">
         <v>11352.77629569</v>
       </c>
-      <c r="Q42" t="n">
-        <v>0</v>
-      </c>
-      <c r="R42" t="n">
-        <v>0</v>
-      </c>
-      <c r="S42" t="n">
-        <v>0</v>
-      </c>
+      <c r="P42" s="6" t="n"/>
+      <c r="Q42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T42" s="6" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" t="n">
+      <c r="A43" s="6" t="n">
         <v>59</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>Trade Republic</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>Core MSCI World USD (Acc)</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E43" s="6" t="inlineStr">
         <is>
           <t>IE00B4L5Y983</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="6" t="inlineStr">
         <is>
           <t>A0RPWH</t>
         </is>
       </c>
-      <c r="G43" t="n">
+      <c r="G43" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H43" s="3" t="n">
+      <c r="H43" s="7" t="n">
         <v>45895</v>
       </c>
-      <c r="I43" t="n">
+      <c r="I43" s="6" t="n">
         <v>104.740071</v>
       </c>
-      <c r="J43" t="n">
+      <c r="J43" s="6" t="n">
         <v>85.94</v>
       </c>
-      <c r="K43" t="n">
+      <c r="K43" s="6" t="n">
         <v>9001.361701739999</v>
       </c>
-      <c r="L43" s="3" t="n">
+      <c r="L43" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M43" t="n">
+      <c r="M43" s="6" t="n">
         <v>104.740071</v>
       </c>
-      <c r="N43" t="n">
+      <c r="N43" s="6" t="n">
         <v>108.46</v>
       </c>
-      <c r="O43" t="n">
+      <c r="O43" s="6" t="n">
         <v>11360.10810066</v>
       </c>
-      <c r="Q43" t="n">
-        <v>0</v>
-      </c>
-      <c r="R43" t="n">
-        <v>0</v>
-      </c>
-      <c r="S43" t="n">
-        <v>0</v>
-      </c>
-      <c r="T43" t="inlineStr">
+      <c r="P43" s="6" t="n"/>
+      <c r="Q43" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R43" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S43" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T43" s="6" t="inlineStr">
         <is>
           <t>Aggiornato Manualmente | PRICE ALERT</t>
         </is>
@@ -3561,142 +3601,144 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="n">
+      <c r="A45" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>Trade Republic</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>Core S&amp;P 500 USD (Acc)</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E45" s="6" t="inlineStr">
         <is>
           <t>IE00B5BMR087</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="6" t="inlineStr">
         <is>
           <t>SXR8.DE</t>
         </is>
       </c>
-      <c r="G45" t="n">
-        <v>1</v>
-      </c>
-      <c r="H45" s="3" t="n">
+      <c r="G45" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H45" s="7" t="n">
         <v>45795</v>
       </c>
-      <c r="I45" t="n">
+      <c r="I45" s="6" t="n">
         <v>19.671873</v>
       </c>
-      <c r="J45" t="n">
+      <c r="J45" s="6" t="n">
         <v>564.62</v>
       </c>
-      <c r="K45" t="n">
+      <c r="K45" s="6" t="n">
         <v>11107.13293326</v>
       </c>
-      <c r="L45" s="3" t="n">
+      <c r="L45" s="7" t="n">
         <v>45931</v>
       </c>
-      <c r="M45" t="n">
+      <c r="M45" s="6" t="n">
         <v>19.671873</v>
       </c>
-      <c r="N45" t="n">
+      <c r="N45" s="6" t="n">
         <v>609.919983</v>
       </c>
-      <c r="O45" t="n">
+      <c r="O45" s="6" t="n">
         <v>11998.26844573816</v>
       </c>
-      <c r="Q45" t="n">
-        <v>0</v>
-      </c>
-      <c r="R45" t="n">
-        <v>0</v>
-      </c>
-      <c r="S45" t="n">
-        <v>0</v>
-      </c>
-      <c r="T45" t="inlineStr">
+      <c r="P45" s="6" t="n"/>
+      <c r="Q45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T45" s="6" t="inlineStr">
         <is>
           <t>Autogestito - TER 0.07% | UPDATED BY AssetMind</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="n">
+      <c r="A46" s="6" t="n">
         <v>60</v>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>Trade Republic</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>Core S&amp;P 500 USD (Acc)</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E46" s="6" t="inlineStr">
         <is>
           <t>IE00B5BMR087</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" s="6" t="inlineStr">
         <is>
           <t>SXR8.DE</t>
         </is>
       </c>
-      <c r="G46" t="n">
-        <v>1</v>
-      </c>
-      <c r="H46" s="3" t="n">
+      <c r="G46" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" s="7" t="n">
         <v>45795</v>
       </c>
-      <c r="I46" t="n">
+      <c r="I46" s="6" t="n">
         <v>19.671873</v>
       </c>
-      <c r="J46" t="n">
+      <c r="J46" s="6" t="n">
         <v>564.62</v>
       </c>
-      <c r="K46" t="n">
+      <c r="K46" s="6" t="n">
         <v>11107.13293326</v>
       </c>
-      <c r="L46" s="3" t="n">
+      <c r="L46" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M46" t="n">
+      <c r="M46" s="6" t="n">
         <v>19.671873</v>
       </c>
-      <c r="N46" t="n">
+      <c r="N46" s="6" t="n">
         <v>611.58</v>
       </c>
-      <c r="O46" t="n">
+      <c r="O46" s="6" t="n">
         <v>12030.92408934</v>
       </c>
-      <c r="Q46" t="n">
-        <v>0</v>
-      </c>
-      <c r="R46" t="n">
-        <v>0</v>
-      </c>
-      <c r="S46" t="n">
-        <v>0</v>
-      </c>
-      <c r="T46" t="inlineStr">
+      <c r="P46" s="6" t="n"/>
+      <c r="Q46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T46" s="6" t="inlineStr">
         <is>
           <t>TER 0.07% | Aggiornato Manualmente - PRICE ALERT</t>
         </is>
@@ -3774,137 +3816,140 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="n">
+      <c r="A48" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>Trade Republic</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="6" t="inlineStr">
         <is>
           <t>S&amp;P 500 Information Tech USD (Acc)</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E48" s="6" t="inlineStr">
         <is>
           <t>IE00B3WJKG14</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" s="6" t="inlineStr">
         <is>
           <t>QDVE.DE</t>
         </is>
       </c>
-      <c r="G48" t="n">
-        <v>1</v>
-      </c>
-      <c r="H48" s="3" t="n">
+      <c r="G48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H48" s="7" t="n">
         <v>45904</v>
       </c>
-      <c r="I48" t="n">
+      <c r="I48" s="6" t="n">
         <v>197.044995</v>
       </c>
-      <c r="J48" t="n">
+      <c r="J48" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="K48" t="n">
+      <c r="K48" s="6" t="n">
         <v>5714.304855</v>
       </c>
-      <c r="L48" s="3" t="n">
+      <c r="L48" s="7" t="n">
         <v>45932</v>
       </c>
-      <c r="M48" t="n">
+      <c r="M48" s="6" t="n">
         <v>197.044995</v>
       </c>
-      <c r="N48" t="n">
+      <c r="N48" s="6" t="n">
         <v>35.46</v>
       </c>
-      <c r="O48" t="n">
+      <c r="O48" s="6" t="n">
         <v>6987.2155227</v>
       </c>
-      <c r="Q48" t="n">
-        <v>0</v>
-      </c>
-      <c r="R48" t="n">
-        <v>0</v>
-      </c>
-      <c r="S48" t="n">
-        <v>0</v>
-      </c>
+      <c r="P48" s="6" t="n"/>
+      <c r="Q48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T48" s="6" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" t="n">
+      <c r="A49" s="6" t="n">
         <v>62</v>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>Trade Republic</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>S&amp;P 500 Information Tech USD (Acc)</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E49" s="6" t="inlineStr">
         <is>
           <t>IE00B3WJKG14</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F49" s="6" t="inlineStr">
         <is>
           <t>QDVE.DE</t>
         </is>
       </c>
-      <c r="G49" t="n">
-        <v>1</v>
-      </c>
-      <c r="H49" s="3" t="n">
+      <c r="G49" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H49" s="7" t="n">
         <v>45904</v>
       </c>
-      <c r="I49" t="n">
+      <c r="I49" s="6" t="n">
         <v>197.044995</v>
       </c>
-      <c r="J49" t="n">
+      <c r="J49" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="K49" t="n">
+      <c r="K49" s="6" t="n">
         <v>5714.304855</v>
       </c>
-      <c r="L49" s="3" t="n">
+      <c r="L49" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M49" t="n">
+      <c r="M49" s="6" t="n">
         <v>220.323194</v>
       </c>
-      <c r="N49" t="n">
+      <c r="N49" s="6" t="n">
         <v>35.16</v>
       </c>
-      <c r="O49" t="n">
+      <c r="O49" s="6" t="n">
         <v>7746.563501039999</v>
       </c>
-      <c r="Q49" t="n">
-        <v>0</v>
-      </c>
-      <c r="R49" t="n">
-        <v>0</v>
-      </c>
-      <c r="S49" t="n">
-        <v>0</v>
-      </c>
-      <c r="T49" t="inlineStr">
+      <c r="P49" s="6" t="n"/>
+      <c r="Q49" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R49" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S49" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T49" s="6" t="inlineStr">
         <is>
           <t>UPDATED BY AssetMind | PRICE ALERT</t>
         </is>
@@ -3982,137 +4027,140 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="n">
+      <c r="A51" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="6" t="inlineStr">
         <is>
           <t>Fondi di investimento</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>Fineco_Adv+</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>BGF World Technology Euro E2</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E51" s="6" t="inlineStr">
         <is>
           <t>LU0171310955</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F51" s="6" t="inlineStr">
         <is>
           <t>MLWTE</t>
         </is>
       </c>
-      <c r="G51" t="n">
+      <c r="G51" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="H51" s="3" t="n">
+      <c r="H51" s="7" t="n">
         <v>45609</v>
       </c>
-      <c r="I51" t="n">
+      <c r="I51" s="6" t="n">
         <v>161.21</v>
       </c>
-      <c r="J51" t="n">
+      <c r="J51" s="6" t="n">
         <v>37.2744</v>
       </c>
-      <c r="K51" t="n">
+      <c r="K51" s="6" t="n">
         <v>6009.006024</v>
       </c>
-      <c r="L51" s="3" t="n">
+      <c r="L51" s="7" t="n">
         <v>45932</v>
       </c>
-      <c r="M51" t="n">
+      <c r="M51" s="6" t="n">
         <v>161.21</v>
       </c>
-      <c r="N51" t="n">
+      <c r="N51" s="6" t="n">
         <v>85.47</v>
       </c>
-      <c r="O51" t="n">
+      <c r="O51" s="6" t="n">
         <v>13778.6187</v>
       </c>
-      <c r="Q51" t="n">
-        <v>0</v>
-      </c>
-      <c r="R51" t="n">
-        <v>0</v>
-      </c>
-      <c r="S51" t="n">
-        <v>0</v>
-      </c>
-      <c r="T51" t="inlineStr">
+      <c r="P51" s="6" t="n"/>
+      <c r="Q51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T51" s="6" t="inlineStr">
         <is>
           <t>PIC</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="n">
+      <c r="A52" s="6" t="n">
         <v>63</v>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="6" t="inlineStr">
         <is>
           <t>Fondi di investimento</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="6" t="inlineStr">
         <is>
           <t>Fineco_Adv+</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" s="6" t="inlineStr">
         <is>
           <t>BGF World Technology Euro E2</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E52" s="6" t="inlineStr">
         <is>
           <t>LU0171310955</t>
         </is>
       </c>
-      <c r="G52" t="n">
+      <c r="F52" s="6" t="n"/>
+      <c r="G52" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="H52" s="3" t="n">
+      <c r="H52" s="7" t="n">
         <v>43662</v>
       </c>
-      <c r="I52" t="n">
+      <c r="I52" s="6" t="n">
         <v>161.21</v>
       </c>
-      <c r="J52" t="n">
+      <c r="J52" s="6" t="n">
         <v>37.2744</v>
       </c>
-      <c r="K52" t="n">
+      <c r="K52" s="6" t="n">
         <v>6009.006024</v>
       </c>
-      <c r="L52" s="3" t="n">
+      <c r="L52" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M52" t="n">
+      <c r="M52" s="6" t="n">
         <v>161.21</v>
       </c>
-      <c r="N52" t="n">
+      <c r="N52" s="6" t="n">
         <v>87.13</v>
       </c>
-      <c r="O52" t="n">
+      <c r="O52" s="6" t="n">
         <v>14046.2273</v>
       </c>
-      <c r="Q52" t="n">
-        <v>0</v>
-      </c>
-      <c r="R52" t="n">
-        <v>0</v>
-      </c>
-      <c r="S52" t="n">
-        <v>0</v>
-      </c>
-      <c r="T52" t="inlineStr">
+      <c r="P52" s="6" t="n"/>
+      <c r="Q52" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R52" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S52" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T52" s="6" t="inlineStr">
         <is>
           <t>PIC | Aggiornato Manualmente</t>
         </is>
@@ -4185,142 +4233,144 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="n">
+      <c r="A54" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="6" t="inlineStr">
         <is>
           <t>Fondi di investimento</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="6" t="inlineStr">
         <is>
           <t>Mediobanca_cons</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" s="6" t="inlineStr">
         <is>
           <t>Nordea 1 – European Covered Bond Opportunities Fund BP</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E54" s="6" t="inlineStr">
         <is>
           <t>LU1915690595</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F54" s="6" t="inlineStr">
         <is>
           <t>NDJX</t>
         </is>
       </c>
-      <c r="G54" t="n">
+      <c r="G54" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H54" s="3" t="n">
+      <c r="H54" s="7" t="n">
         <v>45610</v>
       </c>
-      <c r="I54" t="n">
+      <c r="I54" s="6" t="n">
         <v>287.496</v>
       </c>
-      <c r="J54" t="n">
+      <c r="J54" s="6" t="n">
         <v>109.5321</v>
       </c>
-      <c r="K54" t="n">
+      <c r="K54" s="6" t="n">
         <v>31490.0406216</v>
       </c>
-      <c r="L54" s="3" t="n">
+      <c r="L54" s="7" t="n">
         <v>45932</v>
       </c>
-      <c r="M54" t="n">
+      <c r="M54" s="6" t="n">
         <v>287.496</v>
       </c>
-      <c r="N54" t="n">
+      <c r="N54" s="6" t="n">
         <v>119.7617</v>
       </c>
-      <c r="O54" t="n">
+      <c r="O54" s="6" t="n">
         <v>34431.0097032</v>
       </c>
-      <c r="Q54" t="n">
-        <v>0</v>
-      </c>
-      <c r="R54" t="n">
-        <v>0</v>
-      </c>
-      <c r="S54" t="n">
-        <v>0</v>
-      </c>
-      <c r="T54" t="inlineStr">
+      <c r="P54" s="6" t="n"/>
+      <c r="Q54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T54" s="6" t="inlineStr">
         <is>
           <t>Virgilio</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="n">
+      <c r="A55" s="6" t="n">
         <v>64</v>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="6" t="inlineStr">
         <is>
           <t>Fondi di investimento</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>Mediobanca_cons</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>Nordea 1 – European Covered Bond Opportunities Fund BP</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="E55" s="6" t="inlineStr">
         <is>
           <t>LU1915690595</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="F55" s="6" t="inlineStr">
         <is>
           <t>NDJX</t>
         </is>
       </c>
-      <c r="G55" t="n">
+      <c r="G55" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H55" s="3" t="n">
+      <c r="H55" s="7" t="n">
         <v>45610</v>
       </c>
-      <c r="I55" t="n">
+      <c r="I55" s="6" t="n">
         <v>287.496</v>
       </c>
-      <c r="J55" t="n">
+      <c r="J55" s="6" t="n">
         <v>109.5321</v>
       </c>
-      <c r="K55" t="n">
+      <c r="K55" s="6" t="n">
         <v>31490.0406216</v>
       </c>
-      <c r="L55" s="3" t="n">
+      <c r="L55" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M55" t="n">
+      <c r="M55" s="6" t="n">
         <v>287.496</v>
       </c>
-      <c r="N55" t="n">
+      <c r="N55" s="6" t="n">
         <v>120.1594</v>
       </c>
-      <c r="O55" t="n">
+      <c r="O55" s="6" t="n">
         <v>34545.3468624</v>
       </c>
-      <c r="Q55" t="n">
-        <v>0</v>
-      </c>
-      <c r="R55" t="n">
-        <v>0</v>
-      </c>
-      <c r="S55" t="n">
-        <v>0</v>
-      </c>
-      <c r="T55" t="inlineStr">
+      <c r="P55" s="6" t="n"/>
+      <c r="Q55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T55" s="6" t="inlineStr">
         <is>
           <t>Virgilio | Aggiornato Manualmente</t>
         </is>
@@ -4398,142 +4448,144 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="n">
+      <c r="A57" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="6" t="inlineStr">
         <is>
           <t>Fondi di investimento</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>Mediobanca_cons</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57" s="6" t="inlineStr">
         <is>
           <t>SISF Strategic Credit B Cap EUR Hdg</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E57" s="6" t="inlineStr">
         <is>
           <t>LU1046235815</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="F57" s="6" t="inlineStr">
         <is>
           <t>Classe BH</t>
         </is>
       </c>
-      <c r="G57" t="n">
+      <c r="G57" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H57" s="3" t="n">
+      <c r="H57" s="7" t="n">
         <v>45610</v>
       </c>
-      <c r="I57" t="n">
+      <c r="I57" s="6" t="n">
         <v>291.27</v>
       </c>
-      <c r="J57" t="n">
+      <c r="J57" s="6" t="n">
         <v>108.1079</v>
       </c>
-      <c r="K57" t="n">
+      <c r="K57" s="6" t="n">
         <v>31488.588033</v>
       </c>
-      <c r="L57" s="3" t="n">
+      <c r="L57" s="7" t="n">
         <v>45932</v>
       </c>
-      <c r="M57" t="n">
+      <c r="M57" s="6" t="n">
         <v>291.27</v>
       </c>
-      <c r="N57" t="n">
+      <c r="N57" s="6" t="n">
         <v>124.1968</v>
       </c>
-      <c r="O57" t="n">
+      <c r="O57" s="6" t="n">
         <v>36174.801936</v>
       </c>
-      <c r="Q57" t="n">
-        <v>0</v>
-      </c>
-      <c r="R57" t="n">
-        <v>0</v>
-      </c>
-      <c r="S57" t="n">
-        <v>0</v>
-      </c>
-      <c r="T57" t="inlineStr">
+      <c r="P57" s="6" t="n"/>
+      <c r="Q57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T57" s="6" t="inlineStr">
         <is>
           <t>Virgilio</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="n">
+      <c r="A58" s="6" t="n">
         <v>65</v>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="6" t="inlineStr">
         <is>
           <t>Fondi di investimento</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="6" t="inlineStr">
         <is>
           <t>Mediobanca_cons</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58" s="6" t="inlineStr">
         <is>
           <t>SISF Strategic Credit B Cap EUR Hdg</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>LU1046235815</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="F58" s="6" t="inlineStr">
         <is>
           <t>Classe BH</t>
         </is>
       </c>
-      <c r="G58" t="n">
+      <c r="G58" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H58" s="3" t="n">
+      <c r="H58" s="7" t="n">
         <v>45610</v>
       </c>
-      <c r="I58" t="n">
+      <c r="I58" s="6" t="n">
         <v>291.27</v>
       </c>
-      <c r="J58" t="n">
+      <c r="J58" s="6" t="n">
         <v>108.1079</v>
       </c>
-      <c r="K58" t="n">
+      <c r="K58" s="6" t="n">
         <v>31488.588033</v>
       </c>
-      <c r="L58" s="3" t="n">
+      <c r="L58" s="7" t="n">
         <v>45933</v>
       </c>
-      <c r="M58" t="n">
+      <c r="M58" s="6" t="n">
         <v>291.27</v>
       </c>
-      <c r="N58" t="n">
+      <c r="N58" s="6" t="n">
         <v>124.197</v>
       </c>
-      <c r="O58" t="n">
+      <c r="O58" s="6" t="n">
         <v>36174.86019</v>
       </c>
-      <c r="Q58" t="n">
-        <v>0</v>
-      </c>
-      <c r="R58" t="n">
-        <v>0</v>
-      </c>
-      <c r="S58" t="n">
-        <v>0</v>
-      </c>
-      <c r="T58" t="inlineStr">
+      <c r="P58" s="6" t="n"/>
+      <c r="Q58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T58" s="6" t="inlineStr">
         <is>
           <t>Virgilio | UPDATED BY AssetMind</t>
         </is>
@@ -4723,60 +4775,64 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="n">
+      <c r="A62" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="6" t="inlineStr">
         <is>
           <t>Immobiliare</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="6" t="inlineStr">
         <is>
           <t>Via M. D. Orlando 14</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D62" s="6" t="inlineStr">
         <is>
           <t>Orlando G_sx</t>
         </is>
       </c>
-      <c r="G62" t="n">
-        <v>1</v>
-      </c>
-      <c r="H62" s="3" t="n">
+      <c r="E62" s="6" t="n"/>
+      <c r="F62" s="6" t="n"/>
+      <c r="G62" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H62" s="7" t="n">
         <v>35447</v>
       </c>
-      <c r="I62" t="n">
-        <v>1</v>
-      </c>
-      <c r="J62" t="n">
+      <c r="I62" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J62" s="6" t="n">
         <v>89864</v>
       </c>
-      <c r="K62" t="n">
+      <c r="K62" s="6" t="n">
         <v>89864</v>
       </c>
-      <c r="L62" s="3" t="n">
+      <c r="L62" s="7" t="n">
         <v>39590</v>
       </c>
-      <c r="M62" t="n">
-        <v>1</v>
-      </c>
-      <c r="N62" t="n">
+      <c r="M62" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N62" s="6" t="n">
         <v>180000</v>
       </c>
-      <c r="O62" t="n">
+      <c r="O62" s="6" t="n">
         <v>180000</v>
       </c>
-      <c r="Q62" t="n">
-        <v>0</v>
-      </c>
-      <c r="R62" t="n">
-        <v>0</v>
-      </c>
-      <c r="S62" t="n">
-        <v>0</v>
-      </c>
+      <c r="P62" s="6" t="n"/>
+      <c r="Q62" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R62" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S62" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T62" s="6" t="n"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -4835,116 +4891,124 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="n">
+      <c r="A64" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="6" t="inlineStr">
         <is>
           <t>Immobiliare</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="6" t="inlineStr">
         <is>
           <t>Via M. D. Orlando 14</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64" s="6" t="inlineStr">
         <is>
           <t>Orlando I_dx</t>
         </is>
       </c>
-      <c r="G64" t="n">
-        <v>1</v>
-      </c>
-      <c r="H64" s="3" t="n">
+      <c r="E64" s="6" t="n"/>
+      <c r="F64" s="6" t="n"/>
+      <c r="G64" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H64" s="7" t="n">
         <v>32524</v>
       </c>
-      <c r="I64" t="n">
-        <v>1</v>
-      </c>
-      <c r="J64" t="n">
+      <c r="I64" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J64" s="6" t="n">
         <v>54590</v>
       </c>
-      <c r="K64" t="n">
+      <c r="K64" s="6" t="n">
         <v>54590</v>
       </c>
-      <c r="L64" s="3" t="n">
+      <c r="L64" s="7" t="n">
         <v>35765</v>
       </c>
-      <c r="M64" t="n">
-        <v>1</v>
-      </c>
-      <c r="N64" t="n">
+      <c r="M64" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N64" s="6" t="n">
         <v>89864</v>
       </c>
-      <c r="O64" t="n">
+      <c r="O64" s="6" t="n">
         <v>89864</v>
       </c>
-      <c r="Q64" t="n">
-        <v>0</v>
-      </c>
-      <c r="R64" t="n">
-        <v>0</v>
-      </c>
-      <c r="S64" t="n">
-        <v>0</v>
-      </c>
+      <c r="P64" s="6" t="n"/>
+      <c r="Q64" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R64" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S64" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T64" s="6" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" t="n">
+      <c r="A65" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B65" s="6" t="inlineStr">
         <is>
           <t>Immobiliare</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="6" t="inlineStr">
         <is>
           <t>Via M. D. Orlando 14</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D65" s="6" t="inlineStr">
         <is>
           <t>Orlando I_dx</t>
         </is>
       </c>
-      <c r="G65" t="n">
-        <v>1</v>
-      </c>
-      <c r="H65" s="3" t="n">
+      <c r="E65" s="6" t="n"/>
+      <c r="F65" s="6" t="n"/>
+      <c r="G65" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H65" s="7" t="n">
         <v>32524</v>
       </c>
-      <c r="I65" t="n">
-        <v>1</v>
-      </c>
-      <c r="J65" t="n">
+      <c r="I65" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J65" s="6" t="n">
         <v>54590</v>
       </c>
-      <c r="K65" t="n">
+      <c r="K65" s="6" t="n">
         <v>54590</v>
       </c>
-      <c r="L65" s="3" t="n">
+      <c r="L65" s="7" t="n">
         <v>39590</v>
       </c>
-      <c r="M65" t="n">
-        <v>1</v>
-      </c>
-      <c r="N65" t="n">
+      <c r="M65" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N65" s="6" t="n">
         <v>180000</v>
       </c>
-      <c r="O65" t="n">
+      <c r="O65" s="6" t="n">
         <v>180000</v>
       </c>
-      <c r="Q65" t="n">
-        <v>0</v>
-      </c>
-      <c r="R65" t="n">
-        <v>0</v>
-      </c>
-      <c r="S65" t="n">
-        <v>0</v>
-      </c>
+      <c r="P65" s="6" t="n"/>
+      <c r="Q65" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R65" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S65" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T65" s="6" t="n"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -5003,116 +5067,124 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="n">
+      <c r="A67" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B67" s="6" t="inlineStr">
         <is>
           <t>Immobiliare</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C67" s="6" t="inlineStr">
         <is>
           <t>Via M. D. Orlando 14</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="D67" s="6" t="inlineStr">
         <is>
           <t>Orlando I_sx</t>
         </is>
       </c>
-      <c r="G67" t="n">
-        <v>1</v>
-      </c>
-      <c r="H67" s="3" t="n">
+      <c r="E67" s="6" t="n"/>
+      <c r="F67" s="6" t="n"/>
+      <c r="G67" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H67" s="7" t="n">
         <v>32524</v>
       </c>
-      <c r="I67" t="n">
-        <v>1</v>
-      </c>
-      <c r="J67" t="n">
+      <c r="I67" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J67" s="6" t="n">
         <v>54590</v>
       </c>
-      <c r="K67" t="n">
+      <c r="K67" s="6" t="n">
         <v>54590</v>
       </c>
-      <c r="L67" s="3" t="n">
+      <c r="L67" s="7" t="n">
         <v>35447</v>
       </c>
-      <c r="M67" t="n">
-        <v>1</v>
-      </c>
-      <c r="N67" t="n">
+      <c r="M67" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N67" s="6" t="n">
         <v>89864</v>
       </c>
-      <c r="O67" t="n">
+      <c r="O67" s="6" t="n">
         <v>89864</v>
       </c>
-      <c r="Q67" t="n">
-        <v>0</v>
-      </c>
-      <c r="R67" t="n">
-        <v>0</v>
-      </c>
-      <c r="S67" t="n">
-        <v>0</v>
-      </c>
+      <c r="P67" s="6" t="n"/>
+      <c r="Q67" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R67" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S67" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T67" s="6" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" t="n">
+      <c r="A68" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B68" s="6" t="inlineStr">
         <is>
           <t>Immobiliare</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C68" s="6" t="inlineStr">
         <is>
           <t>Via M. D. Orlando 14</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr">
+      <c r="D68" s="6" t="inlineStr">
         <is>
           <t>Orlando I_sx</t>
         </is>
       </c>
-      <c r="G68" t="n">
-        <v>1</v>
-      </c>
-      <c r="H68" s="3" t="n">
+      <c r="E68" s="6" t="n"/>
+      <c r="F68" s="6" t="n"/>
+      <c r="G68" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H68" s="7" t="n">
         <v>32524</v>
       </c>
-      <c r="I68" t="n">
-        <v>1</v>
-      </c>
-      <c r="J68" t="n">
+      <c r="I68" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J68" s="6" t="n">
         <v>54590</v>
       </c>
-      <c r="K68" t="n">
+      <c r="K68" s="6" t="n">
         <v>54590</v>
       </c>
-      <c r="L68" s="3" t="n">
+      <c r="L68" s="7" t="n">
         <v>39590</v>
       </c>
-      <c r="M68" t="n">
-        <v>1</v>
-      </c>
-      <c r="N68" t="n">
+      <c r="M68" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N68" s="6" t="n">
         <v>180000</v>
       </c>
-      <c r="O68" t="n">
+      <c r="O68" s="6" t="n">
         <v>180000</v>
       </c>
-      <c r="Q68" t="n">
-        <v>0</v>
-      </c>
-      <c r="R68" t="n">
-        <v>0</v>
-      </c>
-      <c r="S68" t="n">
-        <v>0</v>
-      </c>
+      <c r="P68" s="6" t="n"/>
+      <c r="Q68" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R68" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S68" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T68" s="6" t="n"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -6136,132 +6208,136 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="n">
+      <c r="A87" s="6" t="n">
         <v>46</v>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B87" s="6" t="inlineStr">
         <is>
           <t>Titoli di stato</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C87" s="6" t="inlineStr">
         <is>
           <t>Mediobanca_cons</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="D87" s="6" t="inlineStr">
         <is>
           <t>BTP SHORT TERM 3,60</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
+      <c r="E87" s="6" t="inlineStr">
         <is>
           <t>IT0005557084</t>
         </is>
       </c>
-      <c r="G87" t="n">
-        <v>1</v>
-      </c>
-      <c r="H87" s="3" t="n">
+      <c r="F87" s="6" t="n"/>
+      <c r="G87" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H87" s="7" t="n">
         <v>45610</v>
       </c>
-      <c r="I87" t="n">
+      <c r="I87" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="J87" t="n">
+      <c r="J87" s="6" t="n">
         <v>99.51819999999999</v>
       </c>
-      <c r="K87" t="n">
+      <c r="K87" s="6" t="n">
         <v>2089.8822</v>
       </c>
-      <c r="L87" s="3" t="n">
+      <c r="L87" s="7" t="n">
         <v>45931</v>
       </c>
-      <c r="M87" t="n">
+      <c r="M87" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="N87" t="n">
+      <c r="N87" s="6" t="n">
         <v>99.51819999999999</v>
       </c>
-      <c r="O87" t="n">
+      <c r="O87" s="6" t="n">
         <v>2089.8822</v>
       </c>
-      <c r="Q87" t="n">
-        <v>0</v>
-      </c>
-      <c r="R87" t="n">
-        <v>0</v>
-      </c>
-      <c r="S87" t="n">
-        <v>0</v>
-      </c>
-      <c r="T87" t="inlineStr">
+      <c r="P87" s="6" t="n"/>
+      <c r="Q87" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R87" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S87" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T87" s="6" t="inlineStr">
         <is>
           <t>Virgilio</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="n">
+      <c r="A88" s="6" t="n">
         <v>47</v>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B88" s="6" t="inlineStr">
         <is>
           <t>Titoli di stato</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
+      <c r="C88" s="6" t="inlineStr">
         <is>
           <t>Mediobanca_cons</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr">
+      <c r="D88" s="6" t="inlineStr">
         <is>
           <t>BTP SHORT TERM 3,60</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
+      <c r="E88" s="6" t="inlineStr">
         <is>
           <t>IT0005557084</t>
         </is>
       </c>
-      <c r="G88" t="n">
-        <v>1</v>
-      </c>
-      <c r="H88" s="3" t="n">
+      <c r="F88" s="6" t="n"/>
+      <c r="G88" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H88" s="7" t="n">
         <v>45610</v>
       </c>
-      <c r="I88" t="n">
+      <c r="I88" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="J88" t="n">
+      <c r="J88" s="6" t="n">
         <v>99.51819999999999</v>
       </c>
-      <c r="K88" t="n">
+      <c r="K88" s="6" t="n">
         <v>2089.8822</v>
       </c>
-      <c r="L88" s="3" t="n">
+      <c r="L88" s="7" t="n">
         <v>45932</v>
       </c>
-      <c r="M88" t="n">
-        <v>0</v>
-      </c>
-      <c r="N88" t="n">
+      <c r="M88" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N88" s="6" t="n">
         <v>99.51819999999999</v>
       </c>
-      <c r="O88" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q88" t="n">
-        <v>0</v>
-      </c>
-      <c r="R88" t="n">
-        <v>0</v>
-      </c>
-      <c r="S88" t="n">
-        <v>0</v>
-      </c>
-      <c r="T88" t="inlineStr">
+      <c r="O88" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P88" s="6" t="n"/>
+      <c r="Q88" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R88" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S88" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T88" s="6" t="inlineStr">
         <is>
           <t>Virgilio</t>
         </is>

</xml_diff>